<commit_message>
Warm golden redesign, product images, layout cleanup
</commit_message>
<xml_diff>
--- a/Documentation/Best For Lists/Best Budget Friendly Pets List.xlsx
+++ b/Documentation/Best For Lists/Best Budget Friendly Pets List.xlsx
@@ -19,7 +19,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="13">
+  <fonts count="14">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -37,6 +37,12 @@
       <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00595959"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="007B6000"/>
       <sz val="10"/>
     </font>
     <font>
@@ -82,7 +88,7 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00999999"/>
-      <sz val="12"/>
+      <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
@@ -96,12 +102,17 @@
       <sz val="12"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFF2CC"/>
+      </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
@@ -150,7 +161,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="26">
+  <cellXfs count="27">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
@@ -161,68 +172,71 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="9" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="11" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="12" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="5" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -588,18 +602,18 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R19"/>
+  <dimension ref="A1:R20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="12" customWidth="1" min="2" max="2"/>
-    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="5" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="32" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
+    <col width="10" customWidth="1" min="5" max="5"/>
+    <col width="9" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="9" customWidth="1" min="8" max="8"/>
+    <col width="10" customWidth="1" min="9" max="9"/>
     <col width="10" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
     <col width="10" customWidth="1" min="12" max="12"/>
@@ -608,7 +622,7 @@
     <col width="10" customWidth="1" min="15" max="15"/>
     <col width="10" customWidth="1" min="16" max="16"/>
     <col width="10" customWidth="1" min="17" max="17"/>
-    <col width="12" customWidth="1" min="18" max="18"/>
+    <col width="40" customWidth="1" min="18" max="18"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -621,1147 +635,1155 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-06-27  |  Filter: one product per Manufacturer × Price Category × Animal Category  |  Tiebreaker: Score → Rating → Visual Contrast → Review Count  |  Products shown: 15  |  Eliminated: 14</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="16" customHeight="1">
+          <t>Generated: 2026-06-27  |  Products shown: 15  |  Eliminated by dedup rule: 14  |  Pre-filter: Price tier equal Budget Friendly  (0 products removed)</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
       <c r="A3" s="3" t="inlineStr">
         <is>
-          <t>Weights applied:</t>
-        </is>
-      </c>
-      <c r="D3" s="4" t="inlineStr">
-        <is>
-          <t>Durability: 10%</t>
-        </is>
-      </c>
-      <c r="E3" s="4" t="inlineStr">
-        <is>
-          <t>Emotional comfort potential: 15%</t>
-        </is>
-      </c>
-      <c r="F3" s="4" t="inlineStr">
-        <is>
-          <t>Maintenance requirements: 10%</t>
-        </is>
-      </c>
-      <c r="G3" s="4" t="inlineStr">
-        <is>
-          <t>Return / gift suitability: 5%</t>
-        </is>
-      </c>
-      <c r="H3" s="4" t="inlineStr">
-        <is>
-          <t>Review strength: 10%</t>
-        </is>
-      </c>
-      <c r="I3" s="4" t="inlineStr">
-        <is>
-          <t>Simplicity of use: 10%</t>
-        </is>
-      </c>
-      <c r="J3" s="4" t="inlineStr">
-        <is>
-          <t>Tactile comfort: 10%</t>
-        </is>
-      </c>
-      <c r="K3" s="4" t="inlineStr">
-        <is>
-          <t>Value for money: 30%</t>
-        </is>
-      </c>
-    </row>
-    <row r="4" ht="30" customHeight="1">
-      <c r="A4" s="5" t="inlineStr">
+          <t>Pre-filter applied (before scoring): Price tier equal Budget Friendly</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="16" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Weights:</t>
+        </is>
+      </c>
+      <c r="D4" s="5" t="inlineStr">
+        <is>
+          <t>durability: 10%</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>emotional comfort potential: 15%</t>
+        </is>
+      </c>
+      <c r="F4" s="5" t="inlineStr">
+        <is>
+          <t>maintenance requirements: 10%</t>
+        </is>
+      </c>
+      <c r="G4" s="5" t="inlineStr">
+        <is>
+          <t>return / gift suitability: 5%</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="inlineStr">
+        <is>
+          <t>review strength: 10%</t>
+        </is>
+      </c>
+      <c r="I4" s="5" t="inlineStr">
+        <is>
+          <t>simplicity of use: 10%</t>
+        </is>
+      </c>
+      <c r="J4" s="5" t="inlineStr">
+        <is>
+          <t>tactile comfort: 10%</t>
+        </is>
+      </c>
+      <c r="K4" s="5" t="inlineStr">
+        <is>
+          <t>value for money: 30%</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="30" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
         <is>
           <t>Rank</t>
         </is>
       </c>
-      <c r="B4" s="5" t="inlineStr">
+      <c r="B5" s="6" t="inlineStr">
         <is>
           <t>Manufacturer</t>
         </is>
       </c>
-      <c r="C4" s="5" t="inlineStr">
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="D4" s="5" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
         <is>
           <t>Price
 Category</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>Animal
 Type</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
         <is>
           <t>Price</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>Rating</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>Reviews</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
         <is>
           <t>Overall
 Score</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="J5" s="6" t="inlineStr">
         <is>
           <t>durability</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="K5" s="6" t="inlineStr">
         <is>
           <t>emotional comfort potential</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="L5" s="6" t="inlineStr">
         <is>
           <t>maintenance requirements</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="M5" s="6" t="inlineStr">
         <is>
           <t>return / gift suitability</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="N5" s="6" t="inlineStr">
         <is>
           <t>review strength</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="O5" s="6" t="inlineStr">
         <is>
           <t>simplicity of use</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="P5" s="6" t="inlineStr">
         <is>
           <t>tactile comfort</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="Q5" s="6" t="inlineStr">
         <is>
           <t>value for money</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="R5" s="6" t="inlineStr">
         <is>
           <t>Notes / Flags</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="45" customHeight="1">
-      <c r="A5" s="6" t="n">
+    <row r="6" ht="45" customHeight="1">
+      <c r="A6" s="7" t="n">
         <v>1</v>
       </c>
-      <c r="B5" s="7" t="inlineStr">
+      <c r="B6" s="8" t="inlineStr">
         <is>
           <t>Joy for All</t>
         </is>
       </c>
-      <c r="C5" s="7" t="inlineStr">
+      <c r="C6" s="8" t="inlineStr">
         <is>
           <t>Companion Pet Cat Orange Tabby</t>
         </is>
       </c>
-      <c r="D5" s="8" t="inlineStr">
+      <c r="D6" s="9" t="inlineStr">
         <is>
           <t>Best Value</t>
         </is>
       </c>
-      <c r="E5" s="8" t="inlineStr">
+      <c r="E6" s="9" t="inlineStr">
         <is>
           <t>Cat</t>
         </is>
       </c>
-      <c r="F5" s="8" t="n">
+      <c r="F6" s="9" t="n">
         <v>159.99</v>
       </c>
-      <c r="G5" s="8" t="n">
+      <c r="G6" s="9" t="n">
         <v>4.5</v>
       </c>
-      <c r="H5" s="8" t="n">
+      <c r="H6" s="9" t="n">
         <v>11640</v>
       </c>
-      <c r="I5" s="9" t="n">
+      <c r="I6" s="10" t="n">
         <v>4.6</v>
       </c>
-      <c r="J5" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="K5" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L5" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="M5" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="N5" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="O5" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="P5" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q5" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="R5" s="7" t="inlineStr">
+      <c r="J6" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K6" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="L6" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="M6" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="N6" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="O6" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="P6" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q6" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="R6" s="8" t="inlineStr">
         <is>
           <t>All Joy for All variants share identical sensor/audio platform. Sound Quality=1 per locked rubric anchor (documented 'loud unrealistic meow', Best Buy reviews). Sound Level Control=5 per rubric anchor (3-position ON/OFF/MUTE switch). Review Strength=5 per verified 4.4/5 stars, 10,000+ Amazon reviews. Visual contrast varies by coat color — scored per variant. Orange tabby coat — higher visual contrast against most furniture. Review Strength=5: 11,640 reviews, 4.5★ (repo data, 2026-06-22).</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="45" customHeight="1">
-      <c r="A6" s="10" t="n">
+    <row r="7" ht="45" customHeight="1">
+      <c r="A7" s="11" t="n">
         <v>2</v>
       </c>
-      <c r="B6" s="11" t="inlineStr">
+      <c r="B7" s="12" t="inlineStr">
         <is>
           <t>Joy for All</t>
         </is>
       </c>
-      <c r="C6" s="11" t="inlineStr">
+      <c r="C7" s="12" t="inlineStr">
         <is>
           <t>Companion Pet Pup Golden</t>
         </is>
       </c>
-      <c r="D6" s="12" t="inlineStr">
+      <c r="D7" s="13" t="inlineStr">
         <is>
           <t>Best Value</t>
         </is>
       </c>
-      <c r="E6" s="12" t="inlineStr">
+      <c r="E7" s="13" t="inlineStr">
         <is>
           <t>Dog</t>
         </is>
       </c>
-      <c r="F6" s="12" t="n">
+      <c r="F7" s="13" t="n">
         <v>179</v>
       </c>
-      <c r="G6" s="12" t="n">
+      <c r="G7" s="13" t="n">
         <v>4.3</v>
       </c>
-      <c r="H6" s="12" t="n">
+      <c r="H7" s="13" t="n">
         <v>5164</v>
       </c>
-      <c r="I6" s="13" t="n">
+      <c r="I7" s="14" t="n">
         <v>4.6</v>
       </c>
-      <c r="J6" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="K6" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="L6" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="M6" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="N6" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="O6" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="P6" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q6" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="R6" s="11" t="inlineStr">
+      <c r="J7" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="K7" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="L7" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="M7" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="N7" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="O7" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="P7" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q7" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="R7" s="12" t="inlineStr">
         <is>
           <t>All Joy for All variants share identical sensor/audio platform. Sound Quality=1 per locked rubric anchor (documented 'loud unrealistic meow', Best Buy reviews). Sound Level Control=5 per rubric anchor (3-position ON/OFF/MUTE switch). Review Strength=5 per verified 4.4/5 stars, 10,000+ Amazon reviews. Visual contrast varies by coat color — scored per variant. Review Strength=5: 5,164 reviews, 4.3★ (repo data, 2026-06-22).</t>
         </is>
       </c>
     </row>
-    <row r="7" ht="45" customHeight="1">
-      <c r="A7" s="6" t="n">
-        <v>3</v>
-      </c>
-      <c r="B7" s="7" t="inlineStr">
+    <row r="8" ht="45" customHeight="1">
+      <c r="A8" s="7" t="n">
+        <v>3</v>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
         <is>
           <t>Chongker</t>
         </is>
       </c>
-      <c r="C7" s="7" t="inlineStr">
+      <c r="C8" s="8" t="inlineStr">
         <is>
           <t>MateCat Pro</t>
         </is>
       </c>
-      <c r="D7" s="8" t="inlineStr">
+      <c r="D8" s="9" t="inlineStr">
         <is>
           <t>Best Value</t>
         </is>
       </c>
-      <c r="E7" s="8" t="inlineStr">
+      <c r="E8" s="9" t="inlineStr">
         <is>
           <t>Cat</t>
         </is>
       </c>
-      <c r="F7" s="8" t="n">
+      <c r="F8" s="9" t="n">
         <v>178</v>
       </c>
-      <c r="G7" s="8" t="n">
+      <c r="G8" s="9" t="n">
         <v>4.6</v>
       </c>
-      <c r="H7" s="8" t="n">
+      <c r="H8" s="9" t="n">
         <v>456</v>
       </c>
-      <c r="I7" s="9" t="n">
+      <c r="I8" s="10" t="n">
         <v>4.15</v>
       </c>
-      <c r="J7" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="K7" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L7" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="M7" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="N7" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="O7" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="P7" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q7" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="R7" s="7" t="inlineStr">
+      <c r="J8" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K8" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="L8" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="M8" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="N8" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="O8" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="P8" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q8" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="R8" s="8" t="inlineStr">
         <is>
           <t>Touch/voice verified via chongker.com product page and instruction manual (manuals.plus). Multi-zone sensors trigger purring/meowing/heartbeat/movement. Voice wake: responds to specific phrases. 180-day warranty per chongker.com. Sound Level Control=5: ON/MUTE/OFF + volume control. Privacy=5 confirmed: no camera, microphone, or WiFi per Product Matrix. Review Strength=3: 456 reviews, 4.6★ (repo data, 2026-06-22).</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="45" customHeight="1">
-      <c r="A8" s="10" t="n">
-        <v>4</v>
-      </c>
-      <c r="B8" s="11" t="inlineStr">
+    <row r="9" ht="45" customHeight="1">
+      <c r="A9" s="11" t="n">
+        <v>4</v>
+      </c>
+      <c r="B9" s="12" t="inlineStr">
         <is>
           <t>Chongker</t>
         </is>
       </c>
-      <c r="C8" s="11" t="inlineStr">
+      <c r="C9" s="12" t="inlineStr">
         <is>
           <t>Percy Robot Cat</t>
         </is>
       </c>
-      <c r="D8" s="12" t="inlineStr">
+      <c r="D9" s="13" t="inlineStr">
         <is>
           <t>Budget Friendly</t>
         </is>
       </c>
-      <c r="E8" s="12" t="inlineStr">
+      <c r="E9" s="13" t="inlineStr">
         <is>
           <t>Cat</t>
         </is>
       </c>
-      <c r="F8" s="12" t="n">
+      <c r="F9" s="13" t="n">
         <v>89</v>
       </c>
-      <c r="G8" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="H8" s="12" t="n">
+      <c r="G9" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="H9" s="13" t="n">
         <v>16</v>
       </c>
-      <c r="I8" s="13" t="n">
+      <c r="I9" s="14" t="n">
         <v>4.05</v>
       </c>
-      <c r="J8" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="K8" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="L8" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="M8" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="N8" s="12" t="n">
+      <c r="J9" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="K9" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="L9" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="M9" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="N9" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="O8" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="P8" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q8" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="R8" s="11" t="inlineStr">
+      <c r="O9" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="P9" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q9" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="R9" s="12" t="inlineStr">
         <is>
           <t>Cat-form Percy model. Assumed feature parity with Percy 1.1 Robotic Dog. Review strength=3: lower cumulative reviews than Percy 1.1. Verify current features against chongker.com Percy Robot Cat listing before publishing. Review Strength=2: 16 reviews, 5★ (repo data, 2026-06-22).</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="45" customHeight="1">
-      <c r="A9" s="6" t="n">
-        <v>5</v>
-      </c>
-      <c r="B9" s="7" t="inlineStr">
+    <row r="10" ht="45" customHeight="1">
+      <c r="A10" s="7" t="n">
+        <v>5</v>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Chongker</t>
         </is>
       </c>
-      <c r="C9" s="7" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Percy 1.1 Robotic Companion Dog</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D10" s="9" t="inlineStr">
         <is>
           <t>Budget Friendly</t>
         </is>
       </c>
-      <c r="E9" s="8" t="inlineStr">
+      <c r="E10" s="9" t="inlineStr">
         <is>
           <t>Dog</t>
         </is>
       </c>
-      <c r="F9" s="8" t="n">
+      <c r="F10" s="9" t="n">
         <v>89</v>
       </c>
-      <c r="G9" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="H9" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="I9" s="14" t="n">
+      <c r="G10" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="I10" s="15" t="n">
         <v>3.95</v>
       </c>
-      <c r="J9" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="K9" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="L9" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="M9" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="N9" s="8" t="n">
+      <c r="J10" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K10" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="L10" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="M10" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="N10" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="O9" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="P9" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q9" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="R9" s="7" t="inlineStr">
+      <c r="O10" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="P10" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q10" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="R10" s="8" t="inlineStr">
         <is>
           <t>Dog-form companion with touch sensors and heartbeat simulation. Weighted design for sensory relief per product documentation and buying-guide review (keyirobot.com). Feature set verified as broadly equivalent to MateCat Pro platform. Privacy=5: no camera or internet per Product Matrix. Product name updated to match repo: 'Percy 1.1 Robotic Companion Dog'. Review Strength=1: only 5 reviews at time of scoring (repo data, 2026-06-22).</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="45" customHeight="1">
-      <c r="A10" s="10" t="n">
+    <row r="11" ht="45" customHeight="1">
+      <c r="A11" s="11" t="n">
         <v>6</v>
       </c>
-      <c r="B10" s="11" t="inlineStr">
+      <c r="B11" s="12" t="inlineStr">
         <is>
           <t>Furby</t>
         </is>
       </c>
-      <c r="C10" s="11" t="inlineStr">
+      <c r="C11" s="12" t="inlineStr">
         <is>
           <t>DJ Furby</t>
         </is>
       </c>
-      <c r="D10" s="12" t="inlineStr">
+      <c r="D11" s="13" t="inlineStr">
         <is>
           <t>Budget Friendly</t>
         </is>
       </c>
-      <c r="E10" s="12" t="inlineStr">
+      <c r="E11" s="13" t="inlineStr">
         <is>
           <t>Robot</t>
         </is>
       </c>
-      <c r="F10" s="12" t="n">
+      <c r="F11" s="13" t="n">
         <v>50.11</v>
       </c>
-      <c r="G10" s="12" t="n">
+      <c r="G11" s="13" t="n">
         <v>4.8</v>
       </c>
-      <c r="H10" s="12" t="n">
+      <c r="H11" s="13" t="n">
         <v>772</v>
       </c>
-      <c r="I10" s="15" t="n">
+      <c r="I11" s="16" t="n">
         <v>3.9</v>
       </c>
-      <c r="J10" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="K10" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="L10" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="M10" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="N10" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="O10" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="P10" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q10" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="R10" s="11" t="inlineStr">
+      <c r="J11" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="K11" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L11" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="M11" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="N11" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="O11" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="P11" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q11" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="R11" s="12" t="inlineStr">
         <is>
           <t>Hasbro 2023 'Hey Furby' — 25th anniversary edition. No app, no WiFi, no Bluetooth confirmed (Official Furby Wiki; IEEE Spectrum). 4x AA batteries. 5 voice-activated modes, 600+ pre-programmed reactions. Sound Level Control=2: no volume adjustment available (documented consumer complaint); only shutdown or mode switching. Brand=5: Hasbro, globally established, 58M+ units sold over 25 years. Review Strength=5: massive lifetime Amazon review volume. Dementia=2: loud/unpredictable, fantastical non-animal appearance — not recommended for memory care. Privacy=5: confirmed no wireless connectivity in 2023 model. IMPORTANT: DJ Furby (2025) is a different model from the Furby 2023 originally scored — elongated 'long oddbody' form factor with DJ/music theme (per Official Furby Wiki). Core feature scores carried over from 2023 Furby as closest available data; verify DJ-specific features (music modes, controls, form factor) before publishing. Review Strength=4: 772 reviews, 4.8★ (repo data, 2026-06-22). Visual contrast likely higher than regular Furby due to distinctive elongated DJ styling.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="45" customHeight="1">
-      <c r="A11" s="6" t="n">
+    <row r="12" ht="45" customHeight="1">
+      <c r="A12" s="7" t="n">
         <v>7</v>
       </c>
-      <c r="B11" s="7" t="inlineStr">
+      <c r="B12" s="8" t="inlineStr">
         <is>
           <t>Perfect Petzzz</t>
         </is>
       </c>
-      <c r="C11" s="7" t="inlineStr">
+      <c r="C12" s="8" t="inlineStr">
         <is>
           <t>Original Black and White Shorthair Cat</t>
         </is>
       </c>
-      <c r="D11" s="8" t="inlineStr">
+      <c r="D12" s="9" t="inlineStr">
         <is>
           <t>Budget Friendly</t>
         </is>
       </c>
-      <c r="E11" s="8" t="inlineStr">
+      <c r="E12" s="9" t="inlineStr">
         <is>
           <t>Cat</t>
         </is>
       </c>
-      <c r="F11" s="8" t="n">
+      <c r="F12" s="9" t="n">
         <v>44.45</v>
       </c>
-      <c r="G11" s="8" t="n">
+      <c r="G12" s="9" t="n">
         <v>4.4</v>
       </c>
-      <c r="H11" s="8" t="n">
+      <c r="H12" s="9" t="n">
         <v>1200</v>
-      </c>
-      <c r="I11" s="14" t="n">
-        <v>3.8</v>
-      </c>
-      <c r="J11" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="K11" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="L11" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="M11" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="N11" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="O11" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="P11" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q11" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="R11" s="7" t="inlineStr">
-        <is>
-          <t>Breathing-only mechanism; no sensors, voice, or touch response. Sound Quality=1 and Sound Level Control=1 — product produces no sounds; scores reflect absence of any sound output (lowest possible score on both scales). Autonomous Interaction=3: breathing runs continuously without user direction. Review strength estimated; recommend manual verification. Black/white coat: high contrast, distinctive visibility. Product name updated: 'Original Black and White Shorthair Cat' per repo. Review Strength=4: 1200 reviews, 4.4★ (repo, 2026-06-22). SOUND QUALITY FLAG: With budget barking dogs=1 and Joy for All=3, Perfect Petzzz (no sounds at all) may need reconsideration — currently 1 pending Tim review.</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="45" customHeight="1">
-      <c r="A12" s="10" t="n">
-        <v>8</v>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>Perfect Petzzz</t>
-        </is>
-      </c>
-      <c r="C12" s="11" t="inlineStr">
-        <is>
-          <t>Original Chocolate Lab</t>
-        </is>
-      </c>
-      <c r="D12" s="12" t="inlineStr">
-        <is>
-          <t>Budget Friendly</t>
-        </is>
-      </c>
-      <c r="E12" s="12" t="inlineStr">
-        <is>
-          <t>Dog</t>
-        </is>
-      </c>
-      <c r="F12" s="12" t="n">
-        <v>44.45</v>
-      </c>
-      <c r="G12" s="12" t="n">
-        <v>4.3</v>
-      </c>
-      <c r="H12" s="12" t="n">
-        <v>553</v>
       </c>
       <c r="I12" s="15" t="n">
         <v>3.8</v>
       </c>
-      <c r="J12" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="K12" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="L12" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="M12" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="N12" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="O12" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="P12" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q12" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="R12" s="11" t="inlineStr">
+      <c r="J12" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K12" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L12" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="M12" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="N12" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="O12" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="P12" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q12" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="R12" s="8" t="inlineStr">
+        <is>
+          <t>Breathing-only mechanism; no sensors, voice, or touch response. Sound Quality=1 and Sound Level Control=1 — product produces no sounds; scores reflect absence of any sound output (lowest possible score on both scales). Autonomous Interaction=3: breathing runs continuously without user direction. Review strength estimated; recommend manual verification. Black/white coat: high contrast, distinctive visibility. Product name updated: 'Original Black and White Shorthair Cat' per repo. Review Strength=4: 1200 reviews, 4.4★ (repo, 2026-06-22). SOUND QUALITY FLAG: With budget barking dogs=1 and Joy for All=3, Perfect Petzzz (no sounds at all) may need reconsideration — currently 1 pending Tim review.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="45" customHeight="1">
+      <c r="A13" s="11" t="n">
+        <v>8</v>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>Perfect Petzzz</t>
+        </is>
+      </c>
+      <c r="C13" s="12" t="inlineStr">
+        <is>
+          <t>Original Chocolate Lab</t>
+        </is>
+      </c>
+      <c r="D13" s="13" t="inlineStr">
+        <is>
+          <t>Budget Friendly</t>
+        </is>
+      </c>
+      <c r="E13" s="13" t="inlineStr">
+        <is>
+          <t>Dog</t>
+        </is>
+      </c>
+      <c r="F13" s="13" t="n">
+        <v>44.45</v>
+      </c>
+      <c r="G13" s="13" t="n">
+        <v>4.3</v>
+      </c>
+      <c r="H13" s="13" t="n">
+        <v>553</v>
+      </c>
+      <c r="I13" s="16" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="J13" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="K13" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L13" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="M13" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="N13" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="O13" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="P13" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q13" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="R13" s="12" t="inlineStr">
         <is>
           <t>Breathing-only mechanism; no sensors, voice, or touch response. Sound Quality=1 and Sound Level Control=1 — product produces no sounds; scores reflect absence of any sound output (lowest possible score on both scales). Autonomous Interaction=3: breathing runs continuously without user direction. Review strength estimated; recommend manual verification. Product name updated: 'Original Chocolate Lab' per repo. Review Strength=4: 553 reviews, 4.3★ (repo, 2026-06-22). SOUND QUALITY FLAG: With budget barking dogs=1 and Joy for All=3, Perfect Petzzz (no sounds at all) may need reconsideration — currently 1 pending Tim review.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="45" customHeight="1">
-      <c r="A13" s="6" t="n">
+    <row r="14" ht="45" customHeight="1">
+      <c r="A14" s="7" t="n">
         <v>9</v>
       </c>
-      <c r="B13" s="7" t="inlineStr">
+      <c r="B14" s="8" t="inlineStr">
         <is>
           <t>Chongker</t>
         </is>
       </c>
-      <c r="C13" s="7" t="inlineStr">
+      <c r="C14" s="8" t="inlineStr">
         <is>
           <t>Breathing Red Panda Plush</t>
         </is>
       </c>
-      <c r="D13" s="8" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>Best Value</t>
         </is>
       </c>
-      <c r="E13" s="8" t="inlineStr">
+      <c r="E14" s="9" t="inlineStr">
         <is>
           <t>Panda</t>
         </is>
       </c>
-      <c r="F13" s="8" t="n">
+      <c r="F14" s="9" t="n">
         <v>119</v>
       </c>
-      <c r="G13" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="H13" s="8" t="n">
+      <c r="G14" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H14" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="I13" s="14" t="n">
+      <c r="I14" s="15" t="n">
         <v>3.7</v>
       </c>
-      <c r="J13" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="K13" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="L13" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="M13" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="N13" s="8" t="n">
+      <c r="J14" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K14" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="L14" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="M14" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="N14" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="O13" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="P13" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="Q13" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="R13" s="7" t="inlineStr">
+      <c r="O14" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="P14" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="Q14" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="R14" s="8" t="inlineStr">
         <is>
           <t>Detailed scoring performed in prior session against original product spec sheet. Review Strength: no verified current Amazon rating found — manual lookup required before publishing. Control accessibility=3: single ear-switch concealed in fur. Noise Sensitivity=5: explicit mute mode, designed to avoid motor noise per manufacturer. Amazon listing confirmed by Tim: https://www.amazon.com/Chongker-Breathing-Soothing-Interactive-Companion/dp/B0F83R6F75 — Amazon automated access blocked; star rating and review count require manual lookup before updating Review Strength score. Review Strength=1: only 2 reviews at time of scoring (repo data, 2026-06-22). Amazon URL confirmed: amazon.com/dp/B0F83R6F75 — automated fetch blocked; verify rating/count manually before next refresh Value for Money forced to 4 by Tim (June 2026) — consistent with other Chongker product family scores. See Product_Feature_Score_Details.xlsx for rationale.</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="45" customHeight="1">
-      <c r="A14" s="10" t="n">
+    <row r="15" ht="45" customHeight="1">
+      <c r="A15" s="11" t="n">
         <v>10</v>
       </c>
-      <c r="B14" s="11" t="inlineStr">
+      <c r="B15" s="12" t="inlineStr">
         <is>
           <t>Ropet</t>
         </is>
       </c>
-      <c r="C14" s="11" t="inlineStr">
+      <c r="C15" s="12" t="inlineStr">
         <is>
           <t>KAMOMO</t>
         </is>
       </c>
-      <c r="D14" s="12" t="inlineStr">
+      <c r="D15" s="13" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="E14" s="12" t="inlineStr">
+      <c r="E15" s="13" t="inlineStr">
         <is>
           <t>Robot</t>
         </is>
       </c>
-      <c r="F14" s="12" t="n">
+      <c r="F15" s="13" t="n">
         <v>349</v>
       </c>
-      <c r="G14" s="12" t="n">
+      <c r="G15" s="13" t="n">
         <v>4.3</v>
       </c>
-      <c r="H14" s="12" t="n">
+      <c r="H15" s="13" t="n">
         <v>17</v>
       </c>
-      <c r="I14" s="15" t="n">
+      <c r="I15" s="16" t="n">
         <v>3.3</v>
       </c>
-      <c r="J14" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="K14" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="L14" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="M14" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="N14" s="12" t="n">
+      <c r="J15" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="K15" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="L15" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="M15" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="N15" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="O14" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="P14" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="Q14" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="R14" s="11" t="inlineStr">
+      <c r="O15" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="P15" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="Q15" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="R15" s="12" t="inlineStr">
         <is>
           <t>Founded 2022; CES 2025 debut; Series A1 funded (Beijing AI Industry Investment Fund). Privacy=3: local offline AI for daily use; photo uploads encrypted on-device before cloud (ropetai.com). 39°C bionic warmth feature unique in this market (verified Amazon B0GTPZ4N4M). Stationary desktop companion — no locomotion (Movement=1). Brand Reliability=3: legitimate but newer; 30-day returns per manufacturer. Review strength=3: growing — recommend re-check as product matures. Review Strength=2: 17 reviews, 4.3★ (repo data, 2026-06-22).</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="45" customHeight="1">
-      <c r="A15" s="6" t="n">
+    <row r="16" ht="45" customHeight="1">
+      <c r="A16" s="7" t="n">
         <v>11</v>
       </c>
-      <c r="B15" s="7" t="inlineStr">
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>Ruko</t>
         </is>
       </c>
-      <c r="C15" s="7" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>18011 Smart Robot Dog</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D16" s="9" t="inlineStr">
         <is>
           <t>Budget Friendly</t>
         </is>
       </c>
-      <c r="E15" s="8" t="inlineStr">
+      <c r="E16" s="9" t="inlineStr">
         <is>
           <t>Dog</t>
         </is>
       </c>
-      <c r="F15" s="8" t="n">
+      <c r="F16" s="9" t="n">
         <v>69.98999999999999</v>
       </c>
-      <c r="G15" s="8" t="n">
+      <c r="G16" s="9" t="n">
         <v>4.4</v>
       </c>
-      <c r="H15" s="8" t="n">
+      <c r="H16" s="9" t="n">
         <v>283</v>
       </c>
-      <c r="I15" s="16" t="n">
+      <c r="I16" s="17" t="n">
         <v>2.85</v>
       </c>
-      <c r="J15" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="K15" s="8" t="n">
+      <c r="J16" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="K16" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="L15" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="M15" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="N15" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="O15" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="P15" s="8" t="n">
+      <c r="L16" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="M16" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="N16" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="O16" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="P16" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="Q15" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="R15" s="7" t="inlineStr">
+      <c r="Q16" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="R16" s="8" t="inlineStr">
         <is>
           <t>Children's programmable toy robot dog with remote/gesture control. No WiFi or app required (infrared remote — Privacy=5). Hard plastic ABS shell, LED facial expressions, walks/spins/dances. 30-day returns, 90-day warranty per Amazon listing (B0FLXCXPHD). Sound Level Control=2: no volume adjustment noted; on/off states only. Dementia=1: remote-controlled, LED face, not a calming companion product. Not recommended for senior care use cases. Review Strength=3: 283 reviews, 4.4★ (repo data, 2026-06-22).</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="45" customHeight="1">
-      <c r="A16" s="10" t="n">
+    <row r="17" ht="45" customHeight="1">
+      <c r="A17" s="11" t="n">
         <v>12</v>
       </c>
-      <c r="B16" s="11" t="inlineStr">
+      <c r="B17" s="12" t="inlineStr">
         <is>
           <t>Loona</t>
         </is>
       </c>
-      <c r="C16" s="11" t="inlineStr">
+      <c r="C17" s="12" t="inlineStr">
         <is>
           <t>Robot Pet Dog</t>
         </is>
       </c>
-      <c r="D16" s="12" t="inlineStr">
+      <c r="D17" s="13" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="E16" s="12" t="inlineStr">
+      <c r="E17" s="13" t="inlineStr">
         <is>
           <t>Dog</t>
         </is>
       </c>
-      <c r="F16" s="12" t="n">
+      <c r="F17" s="13" t="n">
         <v>499</v>
       </c>
-      <c r="G16" s="12" t="n">
+      <c r="G17" s="13" t="n">
         <v>4.2</v>
       </c>
-      <c r="H16" s="12" t="n">
+      <c r="H17" s="13" t="n">
         <v>1199</v>
       </c>
-      <c r="I16" s="17" t="n">
+      <c r="I17" s="18" t="n">
         <v>2.8</v>
       </c>
-      <c r="J16" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="K16" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="L16" s="12" t="n">
+      <c r="J17" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="K17" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="L17" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="M16" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="N16" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="O16" s="12" t="n">
+      <c r="M17" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="N17" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="O17" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="P16" s="12" t="n">
+      <c r="P17" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="Q16" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="R16" s="11" t="inlineStr">
+      <c r="Q17" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="R17" s="12" t="inlineStr">
         <is>
           <t>KEYi Tech Loona. Rubric anchor product: Control Accessibility=1 (worst) and Customization Options=5 (best). ChatGPT-4o integration. Camera, WiFi, app, account all required. Camera=yes, Internet Access=yes per Product Matrix. Voice=4: excellent AI voice response but conversational not animal-mimicry. Not recommended for seniors or dementia care. Review Strength=4: 1,199 reviews, 4.2★ (repo data, 2026-06-22).</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="45" customHeight="1">
-      <c r="A17" s="6" t="n">
+    <row r="18" ht="45" customHeight="1">
+      <c r="A18" s="7" t="n">
         <v>13</v>
       </c>
-      <c r="B17" s="7" t="inlineStr">
+      <c r="B18" s="8" t="inlineStr">
         <is>
           <t>Wuffy</t>
         </is>
       </c>
-      <c r="C17" s="7" t="inlineStr">
+      <c r="C18" s="8" t="inlineStr">
         <is>
           <t>Wuffy Robot Puppy</t>
         </is>
       </c>
-      <c r="D17" s="8" t="inlineStr">
+      <c r="D18" s="9" t="inlineStr">
         <is>
           <t>Budget Friendly</t>
         </is>
       </c>
-      <c r="E17" s="8" t="inlineStr">
+      <c r="E18" s="9" t="inlineStr">
         <is>
           <t>Dog</t>
         </is>
       </c>
-      <c r="F17" s="8" t="n">
+      <c r="F18" s="9" t="n">
         <v>25.99</v>
       </c>
-      <c r="G17" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="H17" s="8" t="n">
+      <c r="G18" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="H18" s="9" t="n">
         <v>80</v>
       </c>
-      <c r="I17" s="16" t="n">
+      <c r="I18" s="17" t="n">
         <v>2.45</v>
       </c>
-      <c r="J17" s="8" t="n">
+      <c r="J18" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="K17" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="L17" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="M17" s="8" t="n">
+      <c r="K18" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="L18" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="M18" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="N17" s="8" t="n">
+      <c r="N18" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="O17" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="P17" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="Q17" s="8" t="n">
+      <c r="O18" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="P18" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="Q18" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="R17" s="7" t="inlineStr">
+      <c r="R18" s="8" t="inlineStr">
         <is>
           <t>WARNING — LOW CONFIDENCE ACROSS ALL SCORES. No verified independent reviews found; all scores based on wuffyrobot.com marketing claims only. Review Strength=1: no verifiable third-party reviews identified. Brand Reliability=2: new/unverifiable brand, no established track record. Return/Gift Suitability=2: return policy unclear from DTC site. Recommend independent verification of product claims before featuring on site. Compare against Puppy Milow profile for scam-risk indicators. Review Strength=2: 80 reviews but only 3★ (repo data, 2026-06-22). Low rating confirms earlier caution flag about product quality/marketing claims.</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="45" customHeight="1">
-      <c r="A18" s="10" t="n">
+    <row r="19" ht="45" customHeight="1">
+      <c r="A19" s="11" t="n">
         <v>14</v>
       </c>
-      <c r="B18" s="11" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>Enabot</t>
         </is>
       </c>
-      <c r="C18" s="11" t="inlineStr">
+      <c r="C19" s="12" t="inlineStr">
         <is>
           <t>ROLA Mini Pet Monitor</t>
         </is>
       </c>
-      <c r="D18" s="12" t="inlineStr">
+      <c r="D19" s="13" t="inlineStr">
         <is>
           <t>Best Value</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E19" s="13" t="inlineStr">
         <is>
           <t>Robot</t>
         </is>
       </c>
-      <c r="F18" s="12" t="n">
+      <c r="F19" s="13" t="n">
         <v>139</v>
       </c>
-      <c r="G18" s="12" t="n">
-        <v>5</v>
-      </c>
-      <c r="H18" s="12" t="n">
+      <c r="G19" s="13" t="n">
+        <v>5</v>
+      </c>
+      <c r="H19" s="13" t="n">
         <v>73</v>
       </c>
-      <c r="I18" s="17" t="n">
+      <c r="I19" s="18" t="n">
         <v>2.4</v>
       </c>
-      <c r="J18" s="12" t="n">
-        <v>4</v>
-      </c>
-      <c r="K18" s="12" t="n">
+      <c r="J19" s="13" t="n">
+        <v>4</v>
+      </c>
+      <c r="K19" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="L18" s="12" t="n">
+      <c r="L19" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="M18" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="N18" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="O18" s="12" t="n">
+      <c r="M19" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="N19" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="O19" s="13" t="n">
         <v>2</v>
       </c>
-      <c r="P18" s="12" t="n">
+      <c r="P19" s="13" t="n">
         <v>1</v>
       </c>
-      <c r="Q18" s="12" t="n">
-        <v>3</v>
-      </c>
-      <c r="R18" s="11" t="inlineStr">
+      <c r="Q19" s="13" t="n">
+        <v>3</v>
+      </c>
+      <c r="R19" s="12" t="inlineStr">
         <is>
           <t>Camera=yes, Internet Access=yes per Product Matrix. Hard-shell rolling security camera robot; not a companion pet. Scores are category-level; minor spec differences between models noted. Review strength and Value estimated — recommend manual Amazon verification. ROLA Mini is the most compact Enabot; Size=5. Charging=4 (dock, but smaller form factor). Product renamed to 'ROLA Mini Pet Monitor'. Review Strength=3: 73 reviews, 5★ (repo data, 2026-06-22).</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="45" customHeight="1">
-      <c r="A19" s="6" t="n">
+    <row r="20" ht="45" customHeight="1">
+      <c r="A20" s="7" t="n">
         <v>15</v>
       </c>
-      <c r="B19" s="7" t="inlineStr">
+      <c r="B20" s="8" t="inlineStr">
         <is>
           <t>Enabot</t>
         </is>
       </c>
-      <c r="C19" s="7" t="inlineStr">
+      <c r="C20" s="8" t="inlineStr">
         <is>
           <t>EBO Air 2 Plus FamilyBot</t>
         </is>
       </c>
-      <c r="D19" s="8" t="inlineStr">
+      <c r="D20" s="9" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="E19" s="8" t="inlineStr">
+      <c r="E20" s="9" t="inlineStr">
         <is>
           <t>Robot</t>
         </is>
       </c>
-      <c r="F19" s="8" t="n">
+      <c r="F20" s="9" t="n">
         <v>359</v>
       </c>
-      <c r="G19" s="8" t="n">
-        <v>5</v>
-      </c>
-      <c r="H19" s="8" t="n">
+      <c r="G20" s="9" t="n">
+        <v>5</v>
+      </c>
+      <c r="H20" s="9" t="n">
         <v>42</v>
       </c>
-      <c r="I19" s="16" t="n">
+      <c r="I20" s="17" t="n">
         <v>2.3</v>
       </c>
-      <c r="J19" s="8" t="n">
-        <v>4</v>
-      </c>
-      <c r="K19" s="8" t="n">
+      <c r="J20" s="9" t="n">
+        <v>4</v>
+      </c>
+      <c r="K20" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="L19" s="8" t="n">
+      <c r="L20" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="M19" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="N19" s="8" t="n">
+      <c r="M20" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="N20" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="O19" s="8" t="n">
+      <c r="O20" s="9" t="n">
         <v>2</v>
       </c>
-      <c r="P19" s="8" t="n">
+      <c r="P20" s="9" t="n">
         <v>1</v>
       </c>
-      <c r="Q19" s="8" t="n">
-        <v>3</v>
-      </c>
-      <c r="R19" s="7" t="inlineStr">
+      <c r="Q20" s="9" t="n">
+        <v>3</v>
+      </c>
+      <c r="R20" s="8" t="inlineStr">
         <is>
           <t>Camera=yes, Internet Access=yes per Product Matrix. Hard-shell rolling security camera robot; not a companion pet. Scores are category-level; minor spec differences between models noted. Review strength and Value estimated — recommend manual Amazon verification. Air 2 Plus has AI chat mode — highest AI tier in Enabot lineup per manufacturer. Product renamed to 'EBO Air 2 Plus FamilyBot'. Review Strength=3: 42 reviews, 5★ (repo data, 2026-06-22).</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="3">
-    <mergeCell ref="A1:O1"/>
-    <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A2:O2"/>
+  <mergeCells count="4">
+    <mergeCell ref="A3:R3"/>
+    <mergeCell ref="A2:R2"/>
+    <mergeCell ref="A4:C4"/>
+    <mergeCell ref="A1:R1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -1787,583 +1809,583 @@
   </cols>
   <sheetData>
     <row r="1" ht="22" customHeight="1">
-      <c r="A1" s="18" t="inlineStr">
-        <is>
-          <t>Eliminated products — Best Budget Friendly Pets  (same Manufacturer × Price Category × Animal Category slot as a higher-scoring product)</t>
+      <c r="A1" s="19" t="inlineStr">
+        <is>
+          <t>Eliminated by dedup rule — Best Budget Friendly Pets  (same Manufacturer x Price Category x Animal Category as a higher-scoring product)</t>
         </is>
       </c>
     </row>
     <row r="2" ht="22" customHeight="1">
-      <c r="A2" s="5" t="inlineStr">
+      <c r="A2" s="6" t="inlineStr">
         <is>
           <t>Manufacturer</t>
         </is>
       </c>
-      <c r="B2" s="5" t="inlineStr">
+      <c r="B2" s="6" t="inlineStr">
         <is>
           <t>Product</t>
         </is>
       </c>
-      <c r="C2" s="5" t="inlineStr">
+      <c r="C2" s="6" t="inlineStr">
         <is>
           <t>Price Category</t>
         </is>
       </c>
-      <c r="D2" s="5" t="inlineStr">
+      <c r="D2" s="6" t="inlineStr">
         <is>
           <t>Animal</t>
         </is>
       </c>
-      <c r="E2" s="5" t="inlineStr">
+      <c r="E2" s="6" t="inlineStr">
         <is>
           <t>Score</t>
         </is>
       </c>
-      <c r="F2" s="5" t="inlineStr">
+      <c r="F2" s="6" t="inlineStr">
         <is>
           <t>Rating</t>
         </is>
       </c>
-      <c r="G2" s="5" t="inlineStr">
+      <c r="G2" s="6" t="inlineStr">
         <is>
           <t>Kept Instead</t>
         </is>
       </c>
-      <c r="H2" s="5" t="inlineStr">
+      <c r="H2" s="6" t="inlineStr">
         <is>
           <t>Reason</t>
         </is>
       </c>
     </row>
     <row r="3" ht="18" customHeight="1">
-      <c r="A3" s="19" t="inlineStr">
+      <c r="A3" s="20" t="inlineStr">
         <is>
           <t>Joy for All</t>
         </is>
       </c>
-      <c r="B3" s="19" t="inlineStr">
+      <c r="B3" s="20" t="inlineStr">
         <is>
           <t>Companion Pet Cat Tuxedo</t>
         </is>
       </c>
-      <c r="C3" s="19" t="inlineStr">
+      <c r="C3" s="20" t="inlineStr">
         <is>
           <t>Best Value</t>
         </is>
       </c>
-      <c r="D3" s="19" t="inlineStr">
+      <c r="D3" s="20" t="inlineStr">
         <is>
           <t>Cat</t>
         </is>
       </c>
-      <c r="E3" s="19" t="n">
+      <c r="E3" s="20" t="n">
         <v>4.6</v>
       </c>
-      <c r="F3" s="19" t="n">
+      <c r="F3" s="20" t="n">
         <v>4.5</v>
       </c>
-      <c r="G3" s="19" t="inlineStr">
+      <c r="G3" s="20" t="inlineStr">
         <is>
           <t>Companion Pet Cat Orange Tabby</t>
         </is>
       </c>
-      <c r="H3" s="19" t="inlineStr">
-        <is>
-          <t>Score=4.60 rating=4.5</t>
+      <c r="H3" s="20" t="inlineStr">
+        <is>
+          <t>score=4.60 rating=4.5</t>
         </is>
       </c>
     </row>
     <row r="4" ht="18" customHeight="1">
-      <c r="A4" s="20" t="inlineStr">
+      <c r="A4" s="21" t="inlineStr">
         <is>
           <t>Joy for All</t>
         </is>
       </c>
-      <c r="B4" s="20" t="inlineStr">
+      <c r="B4" s="21" t="inlineStr">
         <is>
           <t>Companion Pet Cat Silver</t>
         </is>
       </c>
-      <c r="C4" s="20" t="inlineStr">
+      <c r="C4" s="21" t="inlineStr">
         <is>
           <t>Best Value</t>
         </is>
       </c>
-      <c r="D4" s="20" t="inlineStr">
+      <c r="D4" s="21" t="inlineStr">
         <is>
           <t>Cat</t>
         </is>
       </c>
-      <c r="E4" s="20" t="n">
+      <c r="E4" s="21" t="n">
         <v>4.6</v>
       </c>
-      <c r="F4" s="20" t="n">
+      <c r="F4" s="21" t="n">
         <v>4.5</v>
       </c>
-      <c r="G4" s="20" t="inlineStr">
+      <c r="G4" s="21" t="inlineStr">
         <is>
           <t>Companion Pet Cat Orange Tabby</t>
         </is>
       </c>
-      <c r="H4" s="20" t="inlineStr">
-        <is>
-          <t>Score=4.60 rating=4.5</t>
+      <c r="H4" s="21" t="inlineStr">
+        <is>
+          <t>score=4.60 rating=4.5</t>
         </is>
       </c>
     </row>
     <row r="5" ht="18" customHeight="1">
-      <c r="A5" s="19" t="inlineStr">
+      <c r="A5" s="20" t="inlineStr">
         <is>
           <t>Joy for All</t>
         </is>
       </c>
-      <c r="B5" s="19" t="inlineStr">
+      <c r="B5" s="20" t="inlineStr">
         <is>
           <t>Companion Pet Pup Freckled</t>
         </is>
       </c>
-      <c r="C5" s="19" t="inlineStr">
+      <c r="C5" s="20" t="inlineStr">
         <is>
           <t>Best Value</t>
         </is>
       </c>
-      <c r="D5" s="19" t="inlineStr">
+      <c r="D5" s="20" t="inlineStr">
         <is>
           <t>Dog</t>
         </is>
       </c>
-      <c r="E5" s="19" t="n">
+      <c r="E5" s="20" t="n">
         <v>4.6</v>
       </c>
-      <c r="F5" s="19" t="n">
+      <c r="F5" s="20" t="n">
         <v>4.3</v>
       </c>
-      <c r="G5" s="19" t="inlineStr">
+      <c r="G5" s="20" t="inlineStr">
         <is>
           <t>Companion Pet Pup Golden</t>
         </is>
       </c>
-      <c r="H5" s="19" t="inlineStr">
-        <is>
-          <t>Score=4.60 rating=4.3</t>
+      <c r="H5" s="20" t="inlineStr">
+        <is>
+          <t>score=4.60 rating=4.3</t>
         </is>
       </c>
     </row>
     <row r="6" ht="18" customHeight="1">
-      <c r="A6" s="20" t="inlineStr">
+      <c r="A6" s="21" t="inlineStr">
         <is>
           <t>Chongker</t>
         </is>
       </c>
-      <c r="B6" s="20" t="inlineStr">
+      <c r="B6" s="21" t="inlineStr">
         <is>
           <t>Breathing Calico Percy 2.0</t>
         </is>
       </c>
-      <c r="C6" s="20" t="inlineStr">
+      <c r="C6" s="21" t="inlineStr">
         <is>
           <t>Best Value</t>
         </is>
       </c>
-      <c r="D6" s="20" t="inlineStr">
+      <c r="D6" s="21" t="inlineStr">
         <is>
           <t>Cat</t>
         </is>
       </c>
-      <c r="E6" s="20" t="n">
+      <c r="E6" s="21" t="n">
         <v>4.05</v>
       </c>
-      <c r="F6" s="20" t="n">
-        <v>5</v>
-      </c>
-      <c r="G6" s="20" t="inlineStr">
+      <c r="F6" s="21" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" s="21" t="inlineStr">
         <is>
           <t>MateCat Pro</t>
         </is>
       </c>
-      <c r="H6" s="20" t="inlineStr">
-        <is>
-          <t>Score=4.05 rating=5</t>
+      <c r="H6" s="21" t="inlineStr">
+        <is>
+          <t>score=4.05 rating=5</t>
         </is>
       </c>
     </row>
     <row r="7" ht="18" customHeight="1">
-      <c r="A7" s="19" t="inlineStr">
+      <c r="A7" s="20" t="inlineStr">
         <is>
           <t>Chongker</t>
         </is>
       </c>
-      <c r="B7" s="19" t="inlineStr">
+      <c r="B7" s="20" t="inlineStr">
         <is>
           <t>MateCat 1.1</t>
         </is>
       </c>
-      <c r="C7" s="19" t="inlineStr">
+      <c r="C7" s="20" t="inlineStr">
         <is>
           <t>Best Value</t>
         </is>
       </c>
-      <c r="D7" s="19" t="inlineStr">
+      <c r="D7" s="20" t="inlineStr">
         <is>
           <t>Cat</t>
         </is>
       </c>
-      <c r="E7" s="19" t="n">
+      <c r="E7" s="20" t="n">
         <v>3.8</v>
       </c>
-      <c r="F7" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="G7" s="19" t="inlineStr">
+      <c r="F7" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="G7" s="20" t="inlineStr">
         <is>
           <t>MateCat Pro</t>
         </is>
       </c>
-      <c r="H7" s="19" t="inlineStr">
-        <is>
-          <t>Score=3.80 rating=4</t>
+      <c r="H7" s="20" t="inlineStr">
+        <is>
+          <t>score=3.80 rating=4</t>
         </is>
       </c>
     </row>
     <row r="8" ht="18" customHeight="1">
-      <c r="A8" s="20" t="inlineStr">
+      <c r="A8" s="21" t="inlineStr">
         <is>
           <t>Perfect Petzzz</t>
         </is>
       </c>
-      <c r="B8" s="20" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>Grey Tabby Cat</t>
         </is>
       </c>
-      <c r="C8" s="20" t="inlineStr">
+      <c r="C8" s="21" t="inlineStr">
         <is>
           <t>Budget Friendly</t>
         </is>
       </c>
-      <c r="D8" s="20" t="inlineStr">
+      <c r="D8" s="21" t="inlineStr">
         <is>
           <t>Cat</t>
         </is>
       </c>
-      <c r="E8" s="20" t="n">
+      <c r="E8" s="21" t="n">
         <v>3.8</v>
       </c>
-      <c r="F8" s="20" t="n">
+      <c r="F8" s="21" t="n">
         <v>4.3</v>
       </c>
-      <c r="G8" s="20" t="inlineStr">
+      <c r="G8" s="21" t="inlineStr">
         <is>
           <t>Original Black and White Shorthair Cat</t>
         </is>
       </c>
-      <c r="H8" s="20" t="inlineStr">
-        <is>
-          <t>Score=3.80 rating=4.3</t>
+      <c r="H8" s="21" t="inlineStr">
+        <is>
+          <t>score=3.80 rating=4.3</t>
         </is>
       </c>
     </row>
     <row r="9" ht="18" customHeight="1">
-      <c r="A9" s="19" t="inlineStr">
+      <c r="A9" s="20" t="inlineStr">
         <is>
           <t>Perfect Petzzz</t>
         </is>
       </c>
-      <c r="B9" s="19" t="inlineStr">
+      <c r="B9" s="20" t="inlineStr">
         <is>
           <t>Original Shih Tzu</t>
         </is>
       </c>
-      <c r="C9" s="19" t="inlineStr">
+      <c r="C9" s="20" t="inlineStr">
         <is>
           <t>Budget Friendly</t>
         </is>
       </c>
-      <c r="D9" s="19" t="inlineStr">
+      <c r="D9" s="20" t="inlineStr">
         <is>
           <t>Dog</t>
         </is>
       </c>
-      <c r="E9" s="19" t="n">
+      <c r="E9" s="20" t="n">
         <v>3.8</v>
       </c>
-      <c r="F9" s="19" t="n">
+      <c r="F9" s="20" t="n">
         <v>4.2</v>
       </c>
-      <c r="G9" s="19" t="inlineStr">
+      <c r="G9" s="20" t="inlineStr">
         <is>
           <t>Original Chocolate Lab</t>
         </is>
       </c>
-      <c r="H9" s="19" t="inlineStr">
-        <is>
-          <t>Score=3.80 rating=4.2</t>
+      <c r="H9" s="20" t="inlineStr">
+        <is>
+          <t>score=3.80 rating=4.2</t>
         </is>
       </c>
     </row>
     <row r="10" ht="18" customHeight="1">
-      <c r="A10" s="20" t="inlineStr">
+      <c r="A10" s="21" t="inlineStr">
         <is>
           <t>Perfect Petzzz</t>
         </is>
       </c>
-      <c r="B10" s="20" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>Original Beagle</t>
         </is>
       </c>
-      <c r="C10" s="20" t="inlineStr">
+      <c r="C10" s="21" t="inlineStr">
         <is>
           <t>Budget Friendly</t>
         </is>
       </c>
-      <c r="D10" s="20" t="inlineStr">
+      <c r="D10" s="21" t="inlineStr">
         <is>
           <t>Dog</t>
         </is>
       </c>
-      <c r="E10" s="20" t="n">
+      <c r="E10" s="21" t="n">
         <v>3.7</v>
       </c>
-      <c r="F10" s="20" t="n">
+      <c r="F10" s="21" t="n">
         <v>4.4</v>
       </c>
-      <c r="G10" s="20" t="inlineStr">
+      <c r="G10" s="21" t="inlineStr">
         <is>
           <t>Original Chocolate Lab</t>
         </is>
       </c>
-      <c r="H10" s="20" t="inlineStr">
-        <is>
-          <t>Score=3.70 rating=4.4</t>
+      <c r="H10" s="21" t="inlineStr">
+        <is>
+          <t>score=3.70 rating=4.4</t>
         </is>
       </c>
     </row>
     <row r="11" ht="18" customHeight="1">
-      <c r="A11" s="19" t="inlineStr">
+      <c r="A11" s="20" t="inlineStr">
         <is>
           <t>Perfect Petzzz</t>
         </is>
       </c>
-      <c r="B11" s="19" t="inlineStr">
+      <c r="B11" s="20" t="inlineStr">
         <is>
           <t>Original Border Collie</t>
         </is>
       </c>
-      <c r="C11" s="19" t="inlineStr">
+      <c r="C11" s="20" t="inlineStr">
         <is>
           <t>Budget Friendly</t>
         </is>
       </c>
-      <c r="D11" s="19" t="inlineStr">
+      <c r="D11" s="20" t="inlineStr">
         <is>
           <t>Dog</t>
         </is>
       </c>
-      <c r="E11" s="19" t="n">
+      <c r="E11" s="20" t="n">
         <v>3.7</v>
       </c>
-      <c r="F11" s="19" t="n">
+      <c r="F11" s="20" t="n">
         <v>4.3</v>
       </c>
-      <c r="G11" s="19" t="inlineStr">
+      <c r="G11" s="20" t="inlineStr">
         <is>
           <t>Original Chocolate Lab</t>
         </is>
       </c>
-      <c r="H11" s="19" t="inlineStr">
-        <is>
-          <t>Score=3.70 rating=4.3</t>
+      <c r="H11" s="20" t="inlineStr">
+        <is>
+          <t>score=3.70 rating=4.3</t>
         </is>
       </c>
     </row>
     <row r="12" ht="18" customHeight="1">
-      <c r="A12" s="20" t="inlineStr">
+      <c r="A12" s="21" t="inlineStr">
         <is>
           <t>Perfect Petzzz</t>
         </is>
       </c>
-      <c r="B12" s="20" t="inlineStr">
+      <c r="B12" s="21" t="inlineStr">
         <is>
           <t>Original Siamese Cat</t>
         </is>
       </c>
-      <c r="C12" s="20" t="inlineStr">
+      <c r="C12" s="21" t="inlineStr">
         <is>
           <t>Budget Friendly</t>
         </is>
       </c>
-      <c r="D12" s="20" t="inlineStr">
+      <c r="D12" s="21" t="inlineStr">
         <is>
           <t>Cat</t>
         </is>
       </c>
-      <c r="E12" s="20" t="n">
+      <c r="E12" s="21" t="n">
         <v>3.6</v>
       </c>
-      <c r="F12" s="20" t="n">
+      <c r="F12" s="21" t="n">
         <v>4.1</v>
       </c>
-      <c r="G12" s="20" t="inlineStr">
+      <c r="G12" s="21" t="inlineStr">
         <is>
           <t>Original Black and White Shorthair Cat</t>
         </is>
       </c>
-      <c r="H12" s="20" t="inlineStr">
-        <is>
-          <t>Score=3.60 rating=4.1</t>
+      <c r="H12" s="21" t="inlineStr">
+        <is>
+          <t>score=3.60 rating=4.1</t>
         </is>
       </c>
     </row>
     <row r="13" ht="18" customHeight="1">
-      <c r="A13" s="19" t="inlineStr">
+      <c r="A13" s="20" t="inlineStr">
         <is>
           <t>Perfect Petzzz</t>
         </is>
       </c>
-      <c r="B13" s="19" t="inlineStr">
+      <c r="B13" s="20" t="inlineStr">
         <is>
           <t>Original Plush White Cat</t>
         </is>
       </c>
-      <c r="C13" s="19" t="inlineStr">
+      <c r="C13" s="20" t="inlineStr">
         <is>
           <t>Budget Friendly</t>
         </is>
       </c>
-      <c r="D13" s="19" t="inlineStr">
+      <c r="D13" s="20" t="inlineStr">
         <is>
           <t>Cat</t>
         </is>
       </c>
-      <c r="E13" s="19" t="n">
+      <c r="E13" s="20" t="n">
         <v>3.6</v>
       </c>
-      <c r="F13" s="19" t="n">
-        <v>4</v>
-      </c>
-      <c r="G13" s="19" t="inlineStr">
+      <c r="F13" s="20" t="n">
+        <v>4</v>
+      </c>
+      <c r="G13" s="20" t="inlineStr">
         <is>
           <t>Original Black and White Shorthair Cat</t>
         </is>
       </c>
-      <c r="H13" s="19" t="inlineStr">
-        <is>
-          <t>Score=3.60 rating=4</t>
+      <c r="H13" s="20" t="inlineStr">
+        <is>
+          <t>score=3.60 rating=4</t>
         </is>
       </c>
     </row>
     <row r="14" ht="18" customHeight="1">
-      <c r="A14" s="20" t="inlineStr">
+      <c r="A14" s="21" t="inlineStr">
         <is>
           <t>Enabot</t>
         </is>
       </c>
-      <c r="B14" s="20" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>EBO Air 2 FamilyBot</t>
         </is>
       </c>
-      <c r="C14" s="20" t="inlineStr">
+      <c r="C14" s="21" t="inlineStr">
         <is>
           <t>Best Value</t>
         </is>
       </c>
-      <c r="D14" s="20" t="inlineStr">
+      <c r="D14" s="21" t="inlineStr">
         <is>
           <t>Robot</t>
         </is>
       </c>
-      <c r="E14" s="20" t="n">
+      <c r="E14" s="21" t="n">
         <v>2.4</v>
       </c>
-      <c r="F14" s="20" t="n">
+      <c r="F14" s="21" t="n">
         <v>4.5</v>
       </c>
-      <c r="G14" s="20" t="inlineStr">
+      <c r="G14" s="21" t="inlineStr">
         <is>
           <t>ROLA Mini Pet Monitor</t>
         </is>
       </c>
-      <c r="H14" s="20" t="inlineStr">
-        <is>
-          <t>Score=2.40 rating=4.5</t>
+      <c r="H14" s="21" t="inlineStr">
+        <is>
+          <t>score=2.40 rating=4.5</t>
         </is>
       </c>
     </row>
     <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="19" t="inlineStr">
+      <c r="A15" s="20" t="inlineStr">
         <is>
           <t>Enabot</t>
         </is>
       </c>
-      <c r="B15" s="19" t="inlineStr">
+      <c r="B15" s="20" t="inlineStr">
         <is>
           <t>EBO Air 2S FamilyBot</t>
         </is>
       </c>
-      <c r="C15" s="19" t="inlineStr">
+      <c r="C15" s="20" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="D15" s="19" t="inlineStr">
+      <c r="D15" s="20" t="inlineStr">
         <is>
           <t>Robot</t>
         </is>
       </c>
-      <c r="E15" s="19" t="n">
+      <c r="E15" s="20" t="n">
         <v>2.3</v>
       </c>
-      <c r="F15" s="19" t="n">
-        <v>5</v>
-      </c>
-      <c r="G15" s="19" t="inlineStr">
+      <c r="F15" s="20" t="n">
+        <v>5</v>
+      </c>
+      <c r="G15" s="20" t="inlineStr">
         <is>
           <t>EBO Air 2 Plus FamilyBot</t>
         </is>
       </c>
-      <c r="H15" s="19" t="inlineStr">
-        <is>
-          <t>Score=2.30 rating=5</t>
+      <c r="H15" s="20" t="inlineStr">
+        <is>
+          <t>score=2.30 rating=5</t>
         </is>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1">
-      <c r="A16" s="20" t="inlineStr">
+      <c r="A16" s="21" t="inlineStr">
         <is>
           <t>Enabot</t>
         </is>
       </c>
-      <c r="B16" s="20" t="inlineStr">
+      <c r="B16" s="21" t="inlineStr">
         <is>
           <t>EBO X FamilyBot</t>
         </is>
       </c>
-      <c r="C16" s="20" t="inlineStr">
+      <c r="C16" s="21" t="inlineStr">
         <is>
           <t>Premium</t>
         </is>
       </c>
-      <c r="D16" s="20" t="inlineStr">
+      <c r="D16" s="21" t="inlineStr">
         <is>
           <t>Robot</t>
         </is>
       </c>
-      <c r="E16" s="20" t="n">
+      <c r="E16" s="21" t="n">
         <v>2.3</v>
       </c>
-      <c r="F16" s="20" t="n">
+      <c r="F16" s="21" t="n">
         <v>4.5</v>
       </c>
-      <c r="G16" s="20" t="inlineStr">
+      <c r="G16" s="21" t="inlineStr">
         <is>
           <t>EBO Air 2 Plus FamilyBot</t>
         </is>
       </c>
-      <c r="H16" s="20" t="inlineStr">
-        <is>
-          <t>Score=2.30 rating=4.5</t>
+      <c r="H16" s="21" t="inlineStr">
+        <is>
+          <t>score=2.30 rating=4.5</t>
         </is>
       </c>
     </row>
@@ -2381,7 +2403,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D11"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
@@ -2391,95 +2413,102 @@
   </cols>
   <sheetData>
     <row r="1" ht="20" customHeight="1">
-      <c r="A1" s="21" t="inlineStr">
+      <c r="A1" s="22" t="inlineStr">
         <is>
           <t>Weights applied — Best Budget Friendly Pets</t>
         </is>
       </c>
     </row>
-    <row r="2" ht="18" customHeight="1">
-      <c r="A2" s="22" t="inlineStr">
+    <row r="2" ht="16" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>Pre-filter: Price tier equal Budget Friendly</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="A3" s="23" t="inlineStr">
         <is>
           <t>Feature (scores-file column)</t>
         </is>
       </c>
-      <c r="B2" s="22" t="inlineStr">
+      <c r="B3" s="23" t="inlineStr">
         <is>
           <t>Weight</t>
         </is>
       </c>
-      <c r="C2" s="22" t="inlineStr">
+      <c r="C3" s="23" t="inlineStr">
         <is>
           <t>What It Measures</t>
         </is>
       </c>
-      <c r="D2" s="22" t="inlineStr">
+      <c r="D3" s="23" t="inlineStr">
         <is>
           <t>Score Type</t>
-        </is>
-      </c>
-    </row>
-    <row r="3" ht="20" customHeight="1">
-      <c r="A3" s="23" t="inlineStr">
-        <is>
-          <t>durability</t>
-        </is>
-      </c>
-      <c r="B3" s="23" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="C3" s="23" t="inlineStr">
-        <is>
-          <t>Tolerates frequent handling, drops, or facility use</t>
-        </is>
-      </c>
-      <c r="D3" s="23" t="inlineStr">
-        <is>
-          <t>1 – 5</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="24" t="inlineStr">
         <is>
+          <t>durability</t>
+        </is>
+      </c>
+      <c r="B4" s="24" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C4" s="24" t="inlineStr">
+        <is>
+          <t>Tolerates frequent handling, drops, or facility use</t>
+        </is>
+      </c>
+      <c r="D4" s="24" t="inlineStr">
+        <is>
+          <t>1 – 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1">
+      <c r="A5" s="25" t="inlineStr">
+        <is>
           <t>emotional comfort potential</t>
         </is>
       </c>
-      <c r="B4" s="24" t="inlineStr">
+      <c r="B5" s="25" t="inlineStr">
         <is>
           <t>15%</t>
         </is>
       </c>
-      <c r="C4" s="24" t="inlineStr">
+      <c r="C5" s="25" t="inlineStr">
         <is>
           <t>Likely to provide calm, comfort, companionship, or reassurance</t>
         </is>
       </c>
-      <c r="D4" s="24" t="inlineStr">
+      <c r="D5" s="25" t="inlineStr">
         <is>
           <t>1 – 5</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="1">
-      <c r="A5" s="23" t="inlineStr">
+    <row r="6" ht="20" customHeight="1">
+      <c r="A6" s="24" t="inlineStr">
         <is>
           <t>maintenance requirements</t>
         </is>
       </c>
-      <c r="B5" s="23" t="inlineStr">
+      <c r="B6" s="24" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C5" s="23" t="inlineStr">
+      <c r="C6" s="24" t="inlineStr">
         <is>
           <t>Batteries, charging, cleaning, software updates, accessories. Includes battery replacement difficulty (moved here from Safety risk).</t>
         </is>
       </c>
-      <c r="D5" s="23" t="inlineStr">
+      <c r="D6" s="24" t="inlineStr">
         <is>
           <t>1 – 5
 (reversed:
@@ -2487,45 +2516,23 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1">
-      <c r="A6" s="24" t="inlineStr">
+    <row r="7" ht="20" customHeight="1">
+      <c r="A7" s="25" t="inlineStr">
         <is>
           <t>return / gift suitability</t>
         </is>
       </c>
-      <c r="B6" s="24" t="inlineStr">
+      <c r="B7" s="25" t="inlineStr">
         <is>
           <t>5%</t>
         </is>
       </c>
-      <c r="C6" s="24" t="inlineStr">
+      <c r="C7" s="25" t="inlineStr">
         <is>
           <t>Clear return policy, easy gifting, low risk if recipient does not engage</t>
         </is>
       </c>
-      <c r="D6" s="24" t="inlineStr">
-        <is>
-          <t>1 – 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="23" t="inlineStr">
-        <is>
-          <t>review strength</t>
-        </is>
-      </c>
-      <c r="B7" s="23" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="C7" s="23" t="inlineStr">
-        <is>
-          <t>Star rating combined with number of reviews</t>
-        </is>
-      </c>
-      <c r="D7" s="23" t="inlineStr">
+      <c r="D7" s="25" t="inlineStr">
         <is>
           <t>1 – 5</t>
         </is>
@@ -2534,42 +2541,42 @@
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="24" t="inlineStr">
         <is>
+          <t>review strength</t>
+        </is>
+      </c>
+      <c r="B8" s="24" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C8" s="24" t="inlineStr">
+        <is>
+          <t>Star rating combined with number of reviews</t>
+        </is>
+      </c>
+      <c r="D8" s="24" t="inlineStr">
+        <is>
+          <t>1 – 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="A9" s="25" t="inlineStr">
+        <is>
           <t>simplicity of use</t>
         </is>
       </c>
-      <c r="B8" s="24" t="inlineStr">
+      <c r="B9" s="25" t="inlineStr">
         <is>
           <t>10%</t>
         </is>
       </c>
-      <c r="C8" s="24" t="inlineStr">
+      <c r="C9" s="25" t="inlineStr">
         <is>
           <t>How easy to use without instructions after setup</t>
         </is>
       </c>
-      <c r="D8" s="24" t="inlineStr">
-        <is>
-          <t>1 – 5</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="A9" s="23" t="inlineStr">
-        <is>
-          <t>tactile comfort</t>
-        </is>
-      </c>
-      <c r="B9" s="23" t="inlineStr">
-        <is>
-          <t>10%</t>
-        </is>
-      </c>
-      <c r="C9" s="23" t="inlineStr">
-        <is>
-          <t>Softness, lap comfort, cuddle value, pleasant feel</t>
-        </is>
-      </c>
-      <c r="D9" s="23" t="inlineStr">
+      <c r="D9" s="25" t="inlineStr">
         <is>
           <t>1 – 5</t>
         </is>
@@ -2578,40 +2585,63 @@
     <row r="10" ht="20" customHeight="1">
       <c r="A10" s="24" t="inlineStr">
         <is>
+          <t>tactile comfort</t>
+        </is>
+      </c>
+      <c r="B10" s="24" t="inlineStr">
+        <is>
+          <t>10%</t>
+        </is>
+      </c>
+      <c r="C10" s="24" t="inlineStr">
+        <is>
+          <t>Softness, lap comfort, cuddle value, pleasant feel</t>
+        </is>
+      </c>
+      <c r="D10" s="24" t="inlineStr">
+        <is>
+          <t>1 – 5</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="20" customHeight="1">
+      <c r="A11" s="25" t="inlineStr">
+        <is>
           <t>value for money</t>
         </is>
       </c>
-      <c r="B10" s="24" t="inlineStr">
+      <c r="B11" s="25" t="inlineStr">
         <is>
           <t>30%</t>
         </is>
       </c>
-      <c r="C10" s="24" t="inlineStr">
+      <c r="C11" s="25" t="inlineStr">
         <is>
           <t>Features, quality, and usefulness relative to price</t>
         </is>
       </c>
-      <c r="D10" s="24" t="inlineStr">
+      <c r="D11" s="25" t="inlineStr">
         <is>
           <t>1 – 5</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="16" customHeight="1">
-      <c r="A11" s="25" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="26" t="inlineStr">
         <is>
           <t>TOTAL</t>
         </is>
       </c>
-      <c r="B11" s="25" t="inlineStr">
+      <c r="B12" s="26" t="inlineStr">
         <is>
           <t>100%</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A1:D1"/>
+    <mergeCell ref="A2:D2"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Regenerate product and Best For data
</commit_message>
<xml_diff>
--- a/Documentation/Best For Lists/Best Budget Friendly Pets List.xlsx
+++ b/Documentation/Best For Lists/Best Budget Friendly Pets List.xlsx
@@ -620,7 +620,7 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Generated: 2026-07-16  |  Products shown: 6  |  Eliminated by dedup rule: 3  |  Pre-filter: Price Category equal Budget Friendly  (20 products removed)</t>
+          <t>Generated: 2026-08-10  |  Products shown: 6  |  Eliminated by dedup rule: 3  |  Pre-filter: Price Category equal Budget Friendly  (20 products removed)</t>
         </is>
       </c>
     </row>
@@ -797,13 +797,13 @@
         </is>
       </c>
       <c r="F6" s="9" t="n">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="G6" s="9" t="n">
         <v>5</v>
       </c>
       <c r="H6" s="9" t="n">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="I6" s="10" t="n">
         <v>3.95</v>
@@ -863,13 +863,13 @@
         </is>
       </c>
       <c r="F7" s="13" t="n">
-        <v>50.11</v>
+        <v>69.98999999999999</v>
       </c>
       <c r="G7" s="13" t="n">
         <v>4.8</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>772</v>
+        <v>1132</v>
       </c>
       <c r="I7" s="14" t="n">
         <v>3.9</v>
@@ -929,13 +929,13 @@
         </is>
       </c>
       <c r="F8" s="9" t="n">
-        <v>89</v>
+        <v>99</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>5</v>
+        <v>4.8</v>
       </c>
       <c r="H8" s="9" t="n">
-        <v>5</v>
+        <v>13</v>
       </c>
       <c r="I8" s="10" t="n">
         <v>3.85</v>
@@ -981,7 +981,7 @@
       </c>
       <c r="C9" s="12" t="inlineStr">
         <is>
-          <t>Grey Tabby Cat</t>
+          <t>Original Chocolate Lab</t>
         </is>
       </c>
       <c r="D9" s="13" t="inlineStr">
@@ -991,7 +991,7 @@
       </c>
       <c r="E9" s="13" t="inlineStr">
         <is>
-          <t>Cat</t>
+          <t>Dog</t>
         </is>
       </c>
       <c r="F9" s="13" t="n">
@@ -1001,7 +1001,7 @@
         <v>4.3</v>
       </c>
       <c r="H9" s="13" t="n">
-        <v>848</v>
+        <v>538</v>
       </c>
       <c r="I9" s="14" t="n">
         <v>3.8</v>
@@ -1032,7 +1032,7 @@
       </c>
       <c r="R9" s="12" t="inlineStr">
         <is>
-          <t>Breathing-only mechanism; no sensors, voice, or touch response. Sound Level Control=1 — no on/off switch or mute (battery must be removed to silence). Autonomous Interaction=3: breathing runs continuously without user direction. Review strength estimated; recommend manual verification. Previously scored as 'Calico Cat' — now matched to 'Grey Tabby Cat' per repo. Verify this is the correct product match before publishing. Review Strength=4: 848 reviews, 4.3★ (repo data, 2026-06-22). SOUND QUALITY UPDATE (2026-07-01, Tim-confirmed): Perfect Petzzz is NOT silent — manufacturer FAQ confirms the breathing mechanism emits sound as normal operation, and multiple Amazon reviews describe a mechanical/grinding noise rather than a soothing breath. Sound Quality rescored from 2 to 2 under the new merged rubric (was previously scored under 'absence of sound = neutral' logic, now scored on actual sound character; net score unchanged at 2, but rationale corrected). Sound appears to vary unit to unit per manufacturer's own FAQ and mixed review reports (some units near-silent/subtle snore, others audibly grinding) — no per-unit review data available to differentiate individual SKUs, so all 8 Perfect Petzzz products scored uniformly at 2 pending any future unit-specific verification. DEMENTIA SUITABILITY EVIDENCE TIER (2026-07-02): Tier D — no dementia-specific evidence found (independent or manufacturer); score reflects general sub-criteria judgment only (simplicity, familiar form, calmness, safety). Capped at 3. Score is provisional pending dementia consultant review. DEMENTIA SUITABILITY RECALCULATED (2026-07-02, Tim-directed methodology): Simplicity=5, Familiar Form=4, Safety=5, Calmness=avg(Sound=2, Behavioral Realism=1)=1.5. Raw average of 4 sub-criteria=3.88, rounded=4, Evidence Tier D cap=3 -&gt; Final=3 (no change). This is a first-pass 'best effort' score pending dementia care consultant review (consultant search in progress as of 2026-07-02). Products in the 'Ai &amp; Robotic Pets' Type category are excluded from memory-care-relevant Best For lists via a separate Type filter in the Best For Weighting Table, independent of this score.</t>
+          <t>Breathing-only mechanism; no sensors, voice, or touch response. Sound Level Control=1 — no on/off switch or mute (battery must be removed to silence). Autonomous Interaction=3: breathing runs continuously without user direction. Review strength estimated; recommend manual verification. Product name updated: 'Original Chocolate Lab' per repo. Review Strength=4: 553 reviews, 4.3★ (repo, 2026-06-22). SOUND QUALITY UPDATE (2026-07-01, Tim-confirmed): Perfect Petzzz is NOT silent — manufacturer FAQ confirms the breathing mechanism emits sound as normal operation, and multiple Amazon reviews describe a mechanical/grinding noise rather than a soothing breath. Sound Quality rescored from 2 to 2 under the new merged rubric (was previously scored under 'absence of sound = neutral' logic, now scored on actual sound character; net score unchanged at 2, but rationale corrected). Sound appears to vary unit to unit per manufacturer's own FAQ and mixed review reports (some units near-silent/subtle snore, others audibly grinding) — no per-unit review data available to differentiate individual SKUs, so all 8 Perfect Petzzz products scored uniformly at 2 pending any future unit-specific verification. DEMENTIA SUITABILITY EVIDENCE TIER (2026-07-02): Tier D — no dementia-specific evidence found (independent or manufacturer); score reflects general sub-criteria judgment only (simplicity, familiar form, calmness, safety). Capped at 3. Score is provisional pending dementia consultant review. DEMENTIA SUITABILITY RECALCULATED (2026-07-02, Tim-directed methodology): Simplicity=5, Familiar Form=4, Safety=5, Calmness=avg(Sound=2, Behavioral Realism=1)=1.5. Raw average of 4 sub-criteria=3.88, rounded=4, Evidence Tier D cap=3 -&gt; Final=3 (no change). This is a first-pass 'best effort' score pending dementia care consultant review (consultant search in progress as of 2026-07-02). Products in the 'Ai &amp; Robotic Pets' Type category are excluded from memory-care-relevant Best For lists via a separate Type filter in the Best For Weighting Table, independent of this score.</t>
         </is>
       </c>
     </row>
@@ -1047,7 +1047,7 @@
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Original Chocolate Lab</t>
+          <t>Grey Tabby Cat</t>
         </is>
       </c>
       <c r="D10" s="9" t="inlineStr">
@@ -1057,17 +1057,17 @@
       </c>
       <c r="E10" s="9" t="inlineStr">
         <is>
-          <t>Dog</t>
+          <t>Cat</t>
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>44.45</v>
+        <v>53.9</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>4.3</v>
+        <v>4.2</v>
       </c>
       <c r="H10" s="9" t="n">
-        <v>553</v>
+        <v>25</v>
       </c>
       <c r="I10" s="10" t="n">
         <v>3.8</v>
@@ -1098,7 +1098,7 @@
       </c>
       <c r="R10" s="8" t="inlineStr">
         <is>
-          <t>Breathing-only mechanism; no sensors, voice, or touch response. Sound Level Control=1 — no on/off switch or mute (battery must be removed to silence). Autonomous Interaction=3: breathing runs continuously without user direction. Review strength estimated; recommend manual verification. Product name updated: 'Original Chocolate Lab' per repo. Review Strength=4: 553 reviews, 4.3★ (repo, 2026-06-22). SOUND QUALITY UPDATE (2026-07-01, Tim-confirmed): Perfect Petzzz is NOT silent — manufacturer FAQ confirms the breathing mechanism emits sound as normal operation, and multiple Amazon reviews describe a mechanical/grinding noise rather than a soothing breath. Sound Quality rescored from 2 to 2 under the new merged rubric (was previously scored under 'absence of sound = neutral' logic, now scored on actual sound character; net score unchanged at 2, but rationale corrected). Sound appears to vary unit to unit per manufacturer's own FAQ and mixed review reports (some units near-silent/subtle snore, others audibly grinding) — no per-unit review data available to differentiate individual SKUs, so all 8 Perfect Petzzz products scored uniformly at 2 pending any future unit-specific verification. DEMENTIA SUITABILITY EVIDENCE TIER (2026-07-02): Tier D — no dementia-specific evidence found (independent or manufacturer); score reflects general sub-criteria judgment only (simplicity, familiar form, calmness, safety). Capped at 3. Score is provisional pending dementia consultant review. DEMENTIA SUITABILITY RECALCULATED (2026-07-02, Tim-directed methodology): Simplicity=5, Familiar Form=4, Safety=5, Calmness=avg(Sound=2, Behavioral Realism=1)=1.5. Raw average of 4 sub-criteria=3.88, rounded=4, Evidence Tier D cap=3 -&gt; Final=3 (no change). This is a first-pass 'best effort' score pending dementia care consultant review (consultant search in progress as of 2026-07-02). Products in the 'Ai &amp; Robotic Pets' Type category are excluded from memory-care-relevant Best For lists via a separate Type filter in the Best For Weighting Table, independent of this score.</t>
+          <t>Breathing-only mechanism; no sensors, voice, or touch response. Sound Level Control=1 — no on/off switch or mute (battery must be removed to silence). Autonomous Interaction=3: breathing runs continuously without user direction. Review strength estimated; recommend manual verification. Previously scored as 'Calico Cat' — now matched to 'Grey Tabby Cat' per repo. Verify this is the correct product match before publishing. Review Strength=4: 848 reviews, 4.3★ (repo data, 2026-06-22). SOUND QUALITY UPDATE (2026-07-01, Tim-confirmed): Perfect Petzzz is NOT silent — manufacturer FAQ confirms the breathing mechanism emits sound as normal operation, and multiple Amazon reviews describe a mechanical/grinding noise rather than a soothing breath. Sound Quality rescored from 2 to 2 under the new merged rubric (was previously scored under 'absence of sound = neutral' logic, now scored on actual sound character; net score unchanged at 2, but rationale corrected). Sound appears to vary unit to unit per manufacturer's own FAQ and mixed review reports (some units near-silent/subtle snore, others audibly grinding) — no per-unit review data available to differentiate individual SKUs, so all 8 Perfect Petzzz products scored uniformly at 2 pending any future unit-specific verification. DEMENTIA SUITABILITY EVIDENCE TIER (2026-07-02): Tier D — no dementia-specific evidence found (independent or manufacturer); score reflects general sub-criteria judgment only (simplicity, familiar form, calmness, safety). Capped at 3. Score is provisional pending dementia consultant review. DEMENTIA SUITABILITY RECALCULATED (2026-07-02, Tim-directed methodology): Simplicity=5, Familiar Form=4, Safety=5, Calmness=avg(Sound=2, Behavioral Realism=1)=1.5. Raw average of 4 sub-criteria=3.88, rounded=4, Evidence Tier D cap=3 -&gt; Final=3 (no change). This is a first-pass 'best effort' score pending dementia care consultant review (consultant search in progress as of 2026-07-02). Products in the 'Ai &amp; Robotic Pets' Type category are excluded from memory-care-relevant Best For lists via a separate Type filter in the Best For Weighting Table, independent of this score.</t>
         </is>
       </c>
     </row>
@@ -1130,10 +1130,10 @@
         <v>69.98999999999999</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>4.4</v>
+        <v>4.5</v>
       </c>
       <c r="H11" s="13" t="n">
-        <v>283</v>
+        <v>346</v>
       </c>
       <c r="I11" s="15" t="n">
         <v>2.85</v>
@@ -1272,7 +1272,7 @@
         <v>3.7</v>
       </c>
       <c r="F3" s="17" t="n">
-        <v>4.3</v>
+        <v>4.4</v>
       </c>
       <c r="G3" s="17" t="inlineStr">
         <is>
@@ -1281,7 +1281,7 @@
       </c>
       <c r="H3" s="17" t="inlineStr">
         <is>
-          <t>score=3.70 rating=4.3</t>
+          <t>score=3.70 rating=4.4</t>
         </is>
       </c>
     </row>
@@ -1293,7 +1293,7 @@
       </c>
       <c r="B4" s="18" t="inlineStr">
         <is>
-          <t>Original Siamese Cat</t>
+          <t>Original Plush White Cat</t>
         </is>
       </c>
       <c r="C4" s="18" t="inlineStr">
@@ -1310,7 +1310,7 @@
         <v>3.6</v>
       </c>
       <c r="F4" s="18" t="n">
-        <v>4.1</v>
+        <v>4.2</v>
       </c>
       <c r="G4" s="18" t="inlineStr">
         <is>
@@ -1319,7 +1319,7 @@
       </c>
       <c r="H4" s="18" t="inlineStr">
         <is>
-          <t>score=3.60 rating=4.1</t>
+          <t>score=3.60 rating=4.2</t>
         </is>
       </c>
     </row>
@@ -1331,7 +1331,7 @@
       </c>
       <c r="B5" s="17" t="inlineStr">
         <is>
-          <t>Original Plush White Cat</t>
+          <t>Original Siamese Cat</t>
         </is>
       </c>
       <c r="C5" s="17" t="inlineStr">
@@ -1348,7 +1348,7 @@
         <v>3.6</v>
       </c>
       <c r="F5" s="17" t="n">
-        <v>4</v>
+        <v>4.1</v>
       </c>
       <c r="G5" s="17" t="inlineStr">
         <is>
@@ -1357,7 +1357,7 @@
       </c>
       <c r="H5" s="17" t="inlineStr">
         <is>
-          <t>score=3.60 rating=4</t>
+          <t>score=3.60 rating=4.1</t>
         </is>
       </c>
     </row>

</xml_diff>